<commit_message>
Direct Write Excel for QC-02 Day 6
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-02.xlsx
+++ b/FM-MN-07_QC-02.xlsx
@@ -1721,7 +1721,11 @@
       <c r="E6" s="10" t="inlineStr"/>
       <c r="F6" s="10" t="inlineStr"/>
       <c r="G6" s="10" t="inlineStr"/>
-      <c r="H6" s="10" t="inlineStr"/>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I6" s="10" t="inlineStr"/>
       <c r="J6" s="10" t="inlineStr"/>
       <c r="K6" s="10" t="inlineStr"/>
@@ -1762,7 +1766,11 @@
       <c r="E7" s="10" t="inlineStr"/>
       <c r="F7" s="10" t="inlineStr"/>
       <c r="G7" s="10" t="inlineStr"/>
-      <c r="H7" s="10" t="inlineStr"/>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I7" s="10" t="inlineStr"/>
       <c r="J7" s="10" t="inlineStr"/>
       <c r="K7" s="10" t="inlineStr"/>
@@ -1803,7 +1811,11 @@
       <c r="E8" s="10" t="inlineStr"/>
       <c r="F8" s="10" t="inlineStr"/>
       <c r="G8" s="10" t="inlineStr"/>
-      <c r="H8" s="10" t="inlineStr"/>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I8" s="10" t="inlineStr"/>
       <c r="J8" s="10" t="inlineStr"/>
       <c r="K8" s="10" t="inlineStr"/>
@@ -1844,7 +1856,11 @@
       <c r="E9" s="10" t="inlineStr"/>
       <c r="F9" s="10" t="inlineStr"/>
       <c r="G9" s="10" t="inlineStr"/>
-      <c r="H9" s="10" t="inlineStr"/>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I9" s="10" t="inlineStr"/>
       <c r="J9" s="10" t="inlineStr"/>
       <c r="K9" s="10" t="inlineStr"/>
@@ -1885,7 +1901,11 @@
       <c r="E10" s="10" t="inlineStr"/>
       <c r="F10" s="10" t="inlineStr"/>
       <c r="G10" s="10" t="inlineStr"/>
-      <c r="H10" s="10" t="inlineStr"/>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I10" s="10" t="inlineStr"/>
       <c r="J10" s="10" t="inlineStr"/>
       <c r="K10" s="10" t="inlineStr"/>
@@ -1920,7 +1940,11 @@
       <c r="E11" s="24" t="inlineStr"/>
       <c r="F11" s="24" t="inlineStr"/>
       <c r="G11" s="24" t="inlineStr"/>
-      <c r="H11" s="24" t="inlineStr"/>
+      <c r="H11" s="25" t="inlineStr">
+        <is>
+          <t>สัมพันธ์ รักวิถี</t>
+        </is>
+      </c>
       <c r="I11" s="24" t="inlineStr"/>
       <c r="J11" s="24" t="inlineStr"/>
       <c r="K11" s="24" t="inlineStr"/>
@@ -2102,8 +2126,8 @@
     <mergeCell ref="H11:H12"/>
     <mergeCell ref="Y11:Y12"/>
     <mergeCell ref="J11:J12"/>
+    <mergeCell ref="P11:P12"/>
     <mergeCell ref="B16:AG16"/>
-    <mergeCell ref="P11:P12"/>
     <mergeCell ref="AG11:AG12"/>
     <mergeCell ref="AB2:AG2"/>
     <mergeCell ref="AC18:AG18"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for QC-02 Day 7
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-02.xlsx
+++ b/FM-MN-07_QC-02.xlsx
@@ -1729,7 +1729,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I6" s="10" t="inlineStr"/>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J6" s="10" t="inlineStr"/>
       <c r="K6" s="10" t="inlineStr"/>
       <c r="L6" s="10" t="inlineStr"/>
@@ -1774,7 +1778,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="I7" s="10" t="inlineStr"/>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="J7" s="10" t="inlineStr"/>
       <c r="K7" s="10" t="inlineStr"/>
       <c r="L7" s="10" t="inlineStr"/>
@@ -1819,7 +1827,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I8" s="10" t="inlineStr"/>
+      <c r="I8" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J8" s="10" t="inlineStr"/>
       <c r="K8" s="10" t="inlineStr"/>
       <c r="L8" s="10" t="inlineStr"/>
@@ -1864,7 +1876,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I9" s="10" t="inlineStr"/>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J9" s="10" t="inlineStr"/>
       <c r="K9" s="10" t="inlineStr"/>
       <c r="L9" s="10" t="inlineStr"/>
@@ -1909,7 +1925,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="I10" s="10" t="inlineStr"/>
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="J10" s="10" t="inlineStr"/>
       <c r="K10" s="10" t="inlineStr"/>
       <c r="L10" s="10" t="inlineStr"/>
@@ -1948,7 +1968,11 @@
           <t>สัมพันธ์ รักวิถี</t>
         </is>
       </c>
-      <c r="I11" s="24" t="inlineStr"/>
+      <c r="I11" s="25" t="inlineStr">
+        <is>
+          <t>สัมพันธ์ รักวิถี</t>
+        </is>
+      </c>
       <c r="J11" s="24" t="inlineStr"/>
       <c r="K11" s="24" t="inlineStr"/>
       <c r="L11" s="24" t="inlineStr"/>
@@ -2133,8 +2157,8 @@
     <mergeCell ref="H11:H12"/>
     <mergeCell ref="Y11:Y12"/>
     <mergeCell ref="J11:J12"/>
+    <mergeCell ref="P11:P12"/>
     <mergeCell ref="B16:AG16"/>
-    <mergeCell ref="P11:P12"/>
     <mergeCell ref="AG11:AG12"/>
     <mergeCell ref="AB2:AG2"/>
     <mergeCell ref="AC18:AG18"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for QC-02 Day 8
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-02.xlsx
+++ b/FM-MN-07_QC-02.xlsx
@@ -1734,7 +1734,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J6" s="10" t="inlineStr"/>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K6" s="10" t="inlineStr"/>
       <c r="L6" s="10" t="inlineStr"/>
       <c r="M6" s="10" t="inlineStr"/>
@@ -1783,7 +1787,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="J7" s="10" t="inlineStr"/>
+      <c r="J7" s="10" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="K7" s="10" t="inlineStr"/>
       <c r="L7" s="10" t="inlineStr"/>
       <c r="M7" s="10" t="inlineStr"/>
@@ -1832,7 +1840,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J8" s="10" t="inlineStr"/>
+      <c r="J8" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K8" s="10" t="inlineStr"/>
       <c r="L8" s="10" t="inlineStr"/>
       <c r="M8" s="10" t="inlineStr"/>
@@ -1881,7 +1893,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J9" s="10" t="inlineStr"/>
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K9" s="10" t="inlineStr"/>
       <c r="L9" s="10" t="inlineStr"/>
       <c r="M9" s="10" t="inlineStr"/>
@@ -1930,7 +1946,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="J10" s="10" t="inlineStr"/>
+      <c r="J10" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K10" s="10" t="inlineStr"/>
       <c r="L10" s="10" t="inlineStr"/>
       <c r="M10" s="10" t="inlineStr"/>
@@ -1973,7 +1993,11 @@
           <t>สัมพันธ์ รักวิถี</t>
         </is>
       </c>
-      <c r="J11" s="24" t="inlineStr"/>
+      <c r="J11" s="25" t="inlineStr">
+        <is>
+          <t>สัมพันธ์ รักวิถี</t>
+        </is>
+      </c>
       <c r="K11" s="24" t="inlineStr"/>
       <c r="L11" s="24" t="inlineStr"/>
       <c r="M11" s="24" t="inlineStr"/>
@@ -2157,8 +2181,8 @@
     <mergeCell ref="H11:H12"/>
     <mergeCell ref="Y11:Y12"/>
     <mergeCell ref="J11:J12"/>
+    <mergeCell ref="B16:AG16"/>
     <mergeCell ref="P11:P12"/>
-    <mergeCell ref="B16:AG16"/>
     <mergeCell ref="AG11:AG12"/>
     <mergeCell ref="AB2:AG2"/>
     <mergeCell ref="AC18:AG18"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for QC-02 Day 10
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-02.xlsx
+++ b/FM-MN-07_QC-02.xlsx
@@ -1740,7 +1740,11 @@
         </is>
       </c>
       <c r="K6" s="10" t="inlineStr"/>
-      <c r="L6" s="10" t="inlineStr"/>
+      <c r="L6" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M6" s="10" t="inlineStr"/>
       <c r="N6" s="10" t="inlineStr"/>
       <c r="O6" s="10" t="inlineStr"/>
@@ -1793,7 +1797,11 @@
         </is>
       </c>
       <c r="K7" s="10" t="inlineStr"/>
-      <c r="L7" s="10" t="inlineStr"/>
+      <c r="L7" s="10" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="M7" s="10" t="inlineStr"/>
       <c r="N7" s="10" t="inlineStr"/>
       <c r="O7" s="10" t="inlineStr"/>
@@ -1846,7 +1854,11 @@
         </is>
       </c>
       <c r="K8" s="10" t="inlineStr"/>
-      <c r="L8" s="10" t="inlineStr"/>
+      <c r="L8" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M8" s="10" t="inlineStr"/>
       <c r="N8" s="10" t="inlineStr"/>
       <c r="O8" s="10" t="inlineStr"/>
@@ -1899,7 +1911,11 @@
         </is>
       </c>
       <c r="K9" s="10" t="inlineStr"/>
-      <c r="L9" s="10" t="inlineStr"/>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M9" s="10" t="inlineStr"/>
       <c r="N9" s="10" t="inlineStr"/>
       <c r="O9" s="10" t="inlineStr"/>
@@ -1952,7 +1968,11 @@
         </is>
       </c>
       <c r="K10" s="10" t="inlineStr"/>
-      <c r="L10" s="10" t="inlineStr"/>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="M10" s="10" t="inlineStr"/>
       <c r="N10" s="10" t="inlineStr"/>
       <c r="O10" s="10" t="inlineStr"/>
@@ -1999,7 +2019,11 @@
         </is>
       </c>
       <c r="K11" s="24" t="inlineStr"/>
-      <c r="L11" s="24" t="inlineStr"/>
+      <c r="L11" s="25" t="inlineStr">
+        <is>
+          <t>สัมพันธ์ รักวิถี</t>
+        </is>
+      </c>
       <c r="M11" s="24" t="inlineStr"/>
       <c r="N11" s="24" t="inlineStr"/>
       <c r="O11" s="24" t="inlineStr"/>
@@ -2181,8 +2205,8 @@
     <mergeCell ref="H11:H12"/>
     <mergeCell ref="Y11:Y12"/>
     <mergeCell ref="J11:J12"/>
+    <mergeCell ref="P11:P12"/>
     <mergeCell ref="B16:AG16"/>
-    <mergeCell ref="P11:P12"/>
     <mergeCell ref="AG11:AG12"/>
     <mergeCell ref="AB2:AG2"/>
     <mergeCell ref="AC18:AG18"/>

</xml_diff>